<commit_message>
Backup completo: Actualiza Excel y archivos procesados
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -436,7 +436,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,7 +629,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20260313.jpeg</t>
+          <t>DEDEFENSR_20260313_2.jpeg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige deducción de suplidores para a.jpeg y b.jpeg con datos reales
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -484,38 +484,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>09/06/2025</t>
+          <t>12/03/2023</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B0 200031616</t>
+          <t>28054</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B0 200031616</t>
+          <t>B0200063868</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>09/07/2025</t>
+          <t>11/04/2023</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>453.05</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>2970</v>
+        <v>15455</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20250609.jpeg</t>
+          <t>CADE_20230312.jpeg</t>
         </is>
       </c>
     </row>
@@ -527,109 +527,109 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10/06/2025</t>
+          <t>09/06/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B0 200031626</t>
+          <t>B0 200031616</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B0 200031626</t>
+          <t>B0 200031616</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>10/07/2025</t>
+          <t>09/07/2025</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>453.05</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>375</v>
+        <v>2970</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20250610.jpeg</t>
+          <t>DEDEFENSR_20250609.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>10/06/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0013665</t>
+          <t>B0 200031626</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B020016858</t>
+          <t>B0 200031626</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>08-04-2026</t>
+          <t>10/07/2025</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>553.5</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>3075</v>
+        <v>375</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260309.jpeg</t>
+          <t>DEDEFENSR_20250610.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>Laboratorio Classic Dental</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>18/02/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>B0 200036745</t>
+          <t>44843</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B0 200036745</t>
+          <t>44843</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>18/02/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>360</v>
+        <v>5000</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20260313_2.jpeg</t>
+          <t>LaClDe_20260218.jpeg</t>
         </is>
       </c>
     </row>
@@ -641,63 +641,139 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>09-03-2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0013724</t>
+          <t>0013665</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>B0200016975</t>
+          <t>B020016858</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>08-04-2026</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>570.6</v>
+        <v>553.5</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>3170</v>
+        <v>3075</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260317.jpeg</t>
+          <t>PUDESPJASR_20260309.jpeg</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n"/>
-      <c r="B7" s="1" t="n"/>
-      <c r="C7" s="1" t="n"/>
-      <c r="D7" s="1" t="n"/>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="1" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B0 200036745</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B0 200036745</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>360</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>DEDEFENSR_20260313_2.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0013724</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B0200016975</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>570.6</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>3170</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260317.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="n"/>
+      <c r="D9" s="1" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="1" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" s="3" t="n">
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" s="3" t="n">
         <v>1577.15</v>
       </c>
-      <c r="G8" s="3" t="n">
-        <v>9950</v>
-      </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="G10" s="3" t="n">
+        <v>30405</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Procesa 11 nuevas facturas con deducción de suplidores verificada
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,17 +426,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,296 +484,448 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAPELLAN DENTAL</t>
+          <t>LEKA SUPPLY DENTAL SRL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12/03/2023</t>
+          <t>23/01/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>28054</t>
+          <t>1561</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B0200063868</t>
+          <t>1561</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>11/04/2023</t>
+          <t>23/01/2026</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>15455</v>
+        <v>500</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CADE_20230312.jpeg</t>
+          <t>LESUDESR_20260123.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>ROCE DENTAL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/06/2025</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B0 200031616</t>
+          <t>00138640</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B0 200031616</t>
+          <t>E310000016820</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>09/07/2025</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>453.05</v>
+        <v>12042</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>2970</v>
+        <v>78942</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20250609.jpeg</t>
+          <t>RODE_20260226.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>FARACH, S.A.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10/06/2025</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>B0 200031626</t>
+          <t>9400239473</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B0 200031626</t>
+          <t>E3100000093855</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10/07/2025</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>342</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>375</v>
+        <v>2375</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20250610.jpeg</t>
+          <t>FASA_20260306.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Laboratorio Classic Dental</t>
+          <t>MIS INC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>44843</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>44843</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>5000</v>
+        <v>240</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>LaClDe_20260218.jpeg</t>
+          <t>MIIN_20260318.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0013665</t>
+          <t>51604</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>B020016858</t>
+          <t>E310000003142</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>08-04-2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>553.5</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>3075</v>
+        <v>6190.8</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260309.jpeg</t>
+          <t>CADE_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B0 200036745</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>B0 200036745</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>26/03/2026</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>360</v>
+        <v>48</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20260313_2.jpeg</t>
+          <t>SIDEIMNADO_20260316.jpeg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>Oscar A. Renta Negron, S.A.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0013724</t>
+          <t>VFR-157856</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>B0200016975</t>
+          <t>E3100000048082</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>570.6</v>
+        <v>194.65</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>3170</v>
+        <v>1201.53</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260317.jpeg</t>
+          <t>OsAReNeSA_20260305.jpeg</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="1" t="n"/>
-      <c r="D9" s="1" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
-      <c r="H9" s="1" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>S&amp;M Dental</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/03/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FACT/100024590</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B01000015101</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>247.78</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>1624.34</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>S&amp;De_20260306.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>FRADENT, SRL</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FC01-180844</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>E3100000018329</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>57.35</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>376</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>FRSR_20260309.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MEDICONA, S.R.L.</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>01912</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B01000015084</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>35.08</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MESR_20260316.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>46484</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>E310000010271</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>134.24</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>880</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>DELOSADESR_20260318.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n"/>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="n"/>
+      <c r="D13" s="1" t="n"/>
+      <c r="E13" s="1" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="1" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" s="3" t="n">
-        <v>1577.15</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>30405</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" s="3" t="n">
+        <v>13053.1</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>92607.67</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Skill ejecutada: 18 facturas procesadas y consolidado Excel actualizado
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -435,8 +435,8 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,410 +522,524 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ROCE DENTAL</t>
+          <t>Laboratorio Classic Dental</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>18/02/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>00138640</t>
+          <t>44843</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>E310000016820</t>
+          <t>44843</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>18/02/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>12042</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>78942</v>
+        <v>5000</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>RODE_20260226.jpeg</t>
+          <t>LaClDe_20260218.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FARACH, S.A.</t>
+          <t>ROCE DENTAL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9400239473</t>
+          <t>00138640</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>E3100000093855</t>
+          <t>E310000016820</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>342</v>
+        <v>12042</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2375</v>
+        <v>78942</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>FASA_20260306.jpeg</t>
+          <t>RODE_20260226.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MIS INC</t>
+          <t>FARACH, S.A.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>9400239473</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>E3100000093855</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>342</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>240</v>
+        <v>2375</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>MIIN_20260318.jpeg</t>
+          <t>FASA_20260306.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAPELLAN DENTAL</t>
+          <t>MIS INC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>51604</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>E310000003142</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>6190.8</v>
+        <v>240</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CADE_20260319.jpeg</t>
+          <t>MIIN_20260318.jpeg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A202602606</t>
+          <t>51604</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A202602606</t>
+          <t>E310000003142</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>26/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>48</v>
+        <v>6190.8</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SIDEIMNADO_20260316.jpeg</t>
+          <t>CADE_20260319_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oscar A. Renta Negron, S.A.</t>
+          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>VFR-157856</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>E3100000048082</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>26/03/2026</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>194.65</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>1201.53</v>
+        <v>48</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>OsAReNeSA_20260305.jpeg</t>
+          <t>SIDEIMNADO_20260316.jpeg</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S&amp;M Dental</t>
+          <t>Oscar A. Renta Negron, S.A.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FACT/100024590</t>
+          <t>VFR-157856</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B01000015101</t>
+          <t>E3100000048082</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>247.78</v>
+        <v>194.65</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>1624.34</v>
+        <v>1201.53</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>S&amp;De_20260306.jpeg</t>
+          <t>OsAReNeSA_20260305.jpeg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FRADENT, SRL</t>
+          <t>S&amp;M Dental</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FC01-180844</t>
+          <t>FACT/100024590</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>E3100000018329</t>
+          <t>B01000015101</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>57.35</v>
+        <v>247.78</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>376</v>
+        <v>1624.34</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>FRSR_20260309.jpeg</t>
+          <t>S&amp;De_20260306.jpeg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MEDICONA, S.R.L.</t>
+          <t>FRADENT, SRL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01912</t>
+          <t>FC01-180844</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>B01000015084</t>
+          <t>E3100000018329</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>35.08</v>
+        <v>57.35</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>230</v>
+        <v>376</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>MESR_20260316.jpeg</t>
+          <t>FRSR_20260309.jpeg</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DE LOS SANTOS DENTAL, SRL</t>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>46484</t>
+          <t>B0 200036745</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>E310000010271</t>
+          <t>B0 200036745</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>134.24</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>880</v>
+        <v>360</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>DELOSADESR_20260318.jpeg</t>
+          <t>DEDEFENSR_20260313_2.jpeg</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n"/>
-      <c r="B13" s="1" t="n"/>
-      <c r="C13" s="1" t="n"/>
-      <c r="D13" s="1" t="n"/>
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="1" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MEDICONA, S.R.L.</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>01912</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>B01000015084</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>35.08</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>MESR_20260316.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0013724</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>B0200016975</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>570.6</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>3170</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260317_1.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>46484</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>E310000010271</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>134.24</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>880</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>DELOSADESR_20260318.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="1" t="n"/>
+      <c r="D16" s="1" t="n"/>
+      <c r="E16" s="1" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="1" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" s="3" t="n">
-        <v>13053.1</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>92607.67</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" s="3" t="n">
+        <v>13623.7</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>101137.67</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Skill ejecutada: Procesado lote numérico 01-11 exitosamente
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -435,7 +435,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -515,531 +515,417 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>LESUDESR_20260123.jpeg</t>
+          <t>LESUDESR_20260123_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Laboratorio Classic Dental</t>
+          <t>ROCE DENTAL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>44843</t>
+          <t>00138640</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>44843</t>
+          <t>E310000016820</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>12042</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>5000</v>
+        <v>78942</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>LaClDe_20260218.jpeg</t>
+          <t>RODE_20260226_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ROCE DENTAL</t>
+          <t>FARACH, S.A.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>00138640</t>
+          <t>9400239473</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>E310000016820</t>
+          <t>E3100000093855</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12042</v>
+        <v>342</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>78942</v>
+        <v>2375</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>RODE_20260226.jpeg</t>
+          <t>FASA_20260306_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FARACH, S.A.</t>
+          <t>MIS INC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>9400239473</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>E3100000093855</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>342</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>2375</v>
+        <v>240</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>FASA_20260306.jpeg</t>
+          <t>MIIN_20260318_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MIS INC</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>51604</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>E310000003142</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>240</v>
+        <v>6190.8</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>MIIN_20260318.jpeg</t>
+          <t>CADE_20260319_2.jpeg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAPELLAN DENTAL</t>
+          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>51604</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>E310000003142</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>26/03/2026</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>6190.8</v>
+        <v>48</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CADE_20260319_1.jpeg</t>
+          <t>SIDEIMNADO_20260316_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
+          <t>Oscar A. Renta Negron, S.A.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A202602606</t>
+          <t>VFR-157856</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>A202602606</t>
+          <t>E3100000048082</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>26/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>194.65</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>48</v>
+        <v>1201.53</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SIDEIMNADO_20260316.jpeg</t>
+          <t>OsAReNeSA_20260305_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Oscar A. Renta Negron, S.A.</t>
+          <t>S&amp;M Dental</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05/03/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>VFR-157856</t>
+          <t>FACT/100024590</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>E3100000048082</t>
+          <t>B01000015101</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>194.65</v>
+        <v>247.78</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>1201.53</v>
+        <v>1624.34</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>OsAReNeSA_20260305.jpeg</t>
+          <t>S&amp;De_20260306_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S&amp;M Dental</t>
+          <t>FRADENT, SRL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FACT/100024590</t>
+          <t>FC01-180844</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B01000015101</t>
+          <t>E3100000018329</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>247.78</v>
+        <v>57.35</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>1624.34</v>
+        <v>376</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>S&amp;De_20260306.jpeg</t>
+          <t>FRSR_20260309_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FRADENT, SRL</t>
+          <t>MEDICONA, S.R.L.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FC01-180844</t>
+          <t>01912</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>E3100000018329</t>
+          <t>B01000015084</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>57.35</v>
+        <v>35.08</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>376</v>
+        <v>230</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>FRSR_20260309.jpeg</t>
+          <t>MESR_20260316_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>B0 200036745</t>
+          <t>46484</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>B0 200036745</t>
+          <t>E310000010271</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>134.24</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>360</v>
+        <v>880</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20260313_2.jpeg</t>
+          <t>DELOSADESR_20260318_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>MEDICONA, S.R.L.</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>16/03/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>01912</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>B01000015084</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>15/04/2026</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>35.08</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>230</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>MESR_20260316.jpeg</t>
-        </is>
-      </c>
+      <c r="A13" s="1" t="n"/>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="n"/>
+      <c r="D13" s="1" t="n"/>
+      <c r="E13" s="1" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="1" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>0013724</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>B0200016975</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>16/04/2026</t>
-        </is>
-      </c>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>570.6</v>
+        <v>13053.1</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>3170</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>PUDESPJASR_20260317_1.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>DE LOS SANTOS DENTAL, SRL</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>18/03/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>46484</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>E310000010271</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>17/04/2026</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>134.24</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>880</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>DELOSADESR_20260318.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n"/>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="1" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" s="3" t="n">
-        <v>13623.7</v>
-      </c>
-      <c r="G17" s="3" t="n">
-        <v>101137.67</v>
-      </c>
-      <c r="H17" t="inlineStr"/>
+        <v>92607.67</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Skill ejecutada: 18 facturas numéricas (01-18) procesadas y sincronizadas
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -435,8 +435,8 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,349 +484,349 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LEKA SUPPLY DENTAL SRL</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>23/01/2026</t>
+          <t>12/03/2023</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1561</t>
+          <t>28054</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1561</t>
+          <t>B0200063868</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>23/01/2026</t>
+          <t>11/04/2023</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>500</v>
+        <v>15455</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>LESUDESR_20260123_1.jpeg</t>
+          <t>CADE_20230312.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ROCE DENTAL</t>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>10/06/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>00138640</t>
+          <t>B0 200031626</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>E310000016820</t>
+          <t>B0 200031626</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>31/12/2025</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>12042</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>78942</v>
+        <v>375</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>RODE_20260226_1.jpeg</t>
+          <t>DEDEFENSR_20250610.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FARACH, S.A.</t>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>09/06/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9400239473</t>
+          <t>B0 200031616</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>E3100000093855</t>
+          <t>B0 200031616</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>31/12/2025</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>342</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2375</v>
+        <v>2970</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>FASA_20260306_1.jpeg</t>
+          <t>DEDEFENSR_20250609.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MIS INC</t>
+          <t>LEKA SUPPLY DENTAL SRL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>23/01/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>1561</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>1561</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>23/01/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>240</v>
+        <v>500</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>MIIN_20260318_1.jpeg</t>
+          <t>LESUDESR_20260123.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAPELLAN DENTAL</t>
+          <t>Laboratorio Classic Dental</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>18/02/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>51604</t>
+          <t>44843</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>E310000003142</t>
+          <t>44843</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>18/02/2026</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>6190.8</v>
+        <v>5000</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CADE_20260319_2.jpeg</t>
+          <t>LaClDe_20260218.jpeg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
+          <t>ROCE DENTAL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A202602606</t>
+          <t>00138640</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A202602606</t>
+          <t>E310000016820</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>26/03/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>12042</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>48</v>
+        <v>78942</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SIDEIMNADO_20260316_1.jpeg</t>
+          <t>RODE_20260226.jpeg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oscar A. Renta Negron, S.A.</t>
+          <t>FARACH, S.A.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05/03/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>VFR-157856</t>
+          <t>9400239473</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>E3100000048082</t>
+          <t>E3100000093855</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>194.65</v>
+        <v>342</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>1201.53</v>
+        <v>2375</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>OsAReNeSA_20260305_1.jpeg</t>
+          <t>FASA_20260306.jpeg</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S&amp;M Dental</t>
+          <t>MIS INC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FACT/100024590</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B01000015101</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>247.78</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>1624.34</v>
+        <v>240</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>S&amp;De_20260306_1.jpeg</t>
+          <t>MIIN_20260318.jpeg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FRADENT, SRL</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FC01-180844</t>
+          <t>51604</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>E3100000018329</t>
+          <t>E310000003142</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>57.35</v>
+        <v>0</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>376</v>
+        <v>6190.8</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>FRSR_20260309_1.jpeg</t>
+          <t>CADE_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MEDICONA, S.R.L.</t>
+          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -836,96 +836,362 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01912</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>B01000015084</t>
+          <t>A202602606</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>26/03/2026</t>
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>35.08</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>230</v>
+        <v>48</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>MESR_20260316_1.jpeg</t>
+          <t>SIDEIMNADO_20260316.jpeg</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DE LOS SANTOS DENTAL, SRL</t>
+          <t>Oscar A. Renta Negron, S.A.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>46484</t>
+          <t>VFR-157856</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>E310000010271</t>
+          <t>E3100000048082</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>134.24</v>
+        <v>194.65</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>880</v>
+        <v>1201.53</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>DELOSADESR_20260318_1.jpeg</t>
+          <t>OsAReNeSA_20260305.jpeg</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n"/>
-      <c r="B13" s="1" t="n"/>
-      <c r="C13" s="1" t="n"/>
-      <c r="D13" s="1" t="n"/>
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="1" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>S&amp;M Dental</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/03/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FACT/100024590</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>B01000015101</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>247.78</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>1624.34</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>S&amp;De_20260306.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>FRADENT, SRL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FC01-180844</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>E3100000018329</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>57.35</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>376</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>FRSR_20260309.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0013665</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>B020016858</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>08-04-2026</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>553.5</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>3075</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260309.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>B0 200036745</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>B0 200036745</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>360</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>DEDEFENSR_20260313.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MEDICONA, S.R.L.</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>01912</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>B01000015084</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>35.08</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>MESR_20260316.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0013724</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>B0200016975</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>570.6</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>3170</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260317.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>46484</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>E310000010271</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>134.24</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>880</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>DELOSADESR_20260318.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+      <c r="E20" s="1" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="1" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" s="3" t="n">
-        <v>13053.1</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>92607.67</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" s="3" t="n">
+        <v>14177.2</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>123012.67</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Skill corregida: Re-mapeo y procesamiento exitoso de facturas con nombres incorrectos
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,16 +426,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="43" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -484,714 +484,334 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAPELLAN DENTAL</t>
+          <t>FARACH, S.A.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12/03/2023</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>28054</t>
+          <t>9400239473</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B0200063868</t>
+          <t>E3100000093855</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>11/04/2023</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>342</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>15455</v>
+        <v>2375</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CADE_20230312.jpeg</t>
+          <t>FASA_20260306.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>MIS INC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10/06/2025</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B0 200031626</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B0 200031626</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>31/12/2025</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20250610.jpeg</t>
+          <t>MIIN_20260318.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09/06/2025</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>B0 200031616</t>
+          <t>51604</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B0 200031616</t>
+          <t>E310000003142</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>31/12/2025</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2970</v>
+        <v>6190.8</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20250609.jpeg</t>
+          <t>CADE_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LEKA SUPPLY DENTAL SRL</t>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23/01/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1561</t>
+          <t>0013665</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1561</t>
+          <t>B0200016858</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>23/01/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>483.56</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>500</v>
+        <v>3075</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>LESUDESR_20260123.jpeg</t>
+          <t>PUDESPJASR_20260309.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Laboratorio Classic Dental</t>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>44843</t>
+          <t>0013724</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>44843</t>
+          <t>B0200016975</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0</v>
+        <v>483.56</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>5000</v>
+        <v>3170</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>LaClDe_20260218.jpeg</t>
+          <t>PUDESPJASR_20260317.jpeg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ROCE DENTAL</t>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>00138640</t>
+          <t>46484</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>E310000016820</t>
+          <t>E310000010271</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>12042</v>
+        <v>134.24</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>78942</v>
+        <v>880</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>RODE_20260226.jpeg</t>
+          <t>DELOSADESR_20260318.jpeg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FARACH, S.A.</t>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9400239473</t>
+          <t>0013744</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>E3100000093855</t>
+          <t>B0200017007</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>342</v>
+        <v>137.29</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>2375</v>
+        <v>2440</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>FASA_20260306.jpeg</t>
+          <t>PUDESPJASR_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MIS INC</t>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>20/03/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>B0200036854</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>B0200036854</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>31/12/2026</t>
         </is>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>240</v>
+        <v>1050</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>MIIN_20260318.jpeg</t>
+          <t>DEDEFENSR_20260320.jpeg</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CAPELLAN DENTAL</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>19/03/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>51604</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>E310000003142</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>19/03/2026</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>6190.8</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>CADE_20260319.jpeg</t>
-        </is>
-      </c>
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="1" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SISTEMAS DE IMPLANTES NACIONAL DOMINICANA</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>16/03/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>A202602606</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>A202602606</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>26/03/2026</t>
-        </is>
-      </c>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>1580.65</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>SIDEIMNADO_20260316.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Oscar A. Renta Negron, S.A.</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>05/03/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>VFR-157856</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>E3100000048082</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>04/04/2026</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>194.65</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>1201.53</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>OsAReNeSA_20260305.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>S&amp;M Dental</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>06/03/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>FACT/100024590</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>B01000015101</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>05/04/2026</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>247.78</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>1624.34</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>S&amp;De_20260306.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>FRADENT, SRL</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>09/03/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>FC01-180844</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>E3100000018329</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>08/04/2026</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>57.35</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>376</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>FRSR_20260309.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>09/03/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>0013665</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>B020016858</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>08-04-2026</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>553.5</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>3075</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>PUDESPJASR_20260309.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>13/03/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>B0 200036745</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>B0 200036745</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>360</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>DEDEFENSR_20260313.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>MEDICONA, S.R.L.</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>16/03/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>01912</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>B01000015084</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>15/04/2026</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>35.08</v>
-      </c>
-      <c r="G17" s="3" t="n">
-        <v>230</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>MESR_20260316.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>0013724</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>B0200016975</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>16/04/2026</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>570.6</v>
-      </c>
-      <c r="G18" s="3" t="n">
-        <v>3170</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>PUDESPJASR_20260317.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>DE LOS SANTOS DENTAL, SRL</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>18/03/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>46484</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>E310000010271</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>17/04/2026</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>134.24</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>880</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>DELOSADESR_20260318.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n"/>
-      <c r="B20" s="1" t="n"/>
-      <c r="C20" s="1" t="n"/>
-      <c r="D20" s="1" t="n"/>
-      <c r="E20" s="1" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="1" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" s="3" t="n">
-        <v>14177.2</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>123012.67</v>
-      </c>
-      <c r="H21" t="inlineStr"/>
+        <v>19420.8</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ajuste de alcance: Visualización por lotes y detección inteligente por palabras clave
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,15 +426,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
@@ -598,220 +598,68 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0013665</t>
+          <t>46484</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B0200016858</t>
+          <t>E310000010271</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>483.56</v>
+        <v>134.24</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>3075</v>
+        <v>880</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260309.jpeg</t>
+          <t>DELOSADESR_20260318.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>0013724</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>B0200016975</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>16/04/2026</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>483.56</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>3170</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>PUDESPJASR_20260317.jpeg</t>
-        </is>
-      </c>
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="1" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DE LOS SANTOS DENTAL, SRL</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>18/03/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>46484</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>E310000010271</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>17/04/2026</t>
-        </is>
-      </c>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>134.24</v>
+        <v>476.24</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>880</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>DELOSADESR_20260318.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>19/03/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0013744</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>B0200017007</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>18/04/2026</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>137.29</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>2440</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>PUDESPJASR_20260319.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>20/03/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>B0200036854</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>B0200036854</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>31/12/2026</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>1050</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>DEDEFENSR_20260320.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="1" t="n"/>
-      <c r="C10" s="1" t="n"/>
-      <c r="D10" s="1" t="n"/>
-      <c r="E10" s="1" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="1" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" s="3" t="n">
-        <v>1580.65</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>19420.8</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
+        <v>9685.799999999999</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Corrección Extrema: Suplidores reales verificados de cada imagen (Depósito Fernández y Punto Dental)
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -598,68 +598,220 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DE LOS SANTOS DENTAL, SRL</t>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>46484</t>
+          <t>0013665</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>E310000010271</t>
+          <t>B0200016858</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>134.24</v>
+        <v>558.22</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>880</v>
+        <v>3075</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DELOSADESR_20260318.jpeg</t>
+          <t>PUDESPJASR_20260309.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n"/>
-      <c r="B6" s="1" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="1" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0013724</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B0200016975</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>483.56</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>3170</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260317.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>46484</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>E310000010271</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>134.24</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>880</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>DELOSADESR_20260318.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0013744</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B0200017007</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>137.29</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>2440</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260319.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B0200036854</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B0200036854</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>1050</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>DEDEFENSR_20260320.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="1" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" s="3" t="n">
-        <v>476.24</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>9685.799999999999</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" s="3" t="n">
+        <v>1655.31</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>19420.8</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Automatización Local: Ocultar botón 'Subir' y conteo automático de archivos
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,13 +426,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -484,182 +484,258 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>12/03/2023</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0013665</t>
+          <t>28054</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B0200016858</t>
+          <t>B0200063868</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>11/04/2023</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>558.22</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>3075</v>
+        <v>15455</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260309.jpeg</t>
+          <t>CADE_20230312_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>FARACH, S.A.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0013724</t>
+          <t>9400239473</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B0200016975</t>
+          <t>E3100000093855</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>483.56</v>
+        <v>342</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>3170</v>
+        <v>2375</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260317.jpeg</t>
+          <t>FASA_20260306.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>MIS INC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0013744</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B0200017007</t>
+          <t>23898</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>137.29</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2440</v>
+        <v>240</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260319.jpeg</t>
+          <t>MIIN_20260318.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>B0200036854</t>
+          <t>51604</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B0200036854</t>
+          <t>E310000003142</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1050</v>
+        <v>6190.8</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DEDEFENSR_20260320.jpeg</t>
+          <t>CADE_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n"/>
-      <c r="B6" s="1" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="1" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MEDICONA, S.R.L.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>01912</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B01000015084</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>35.08</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>MESR_20260316.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>DE LOS SANTOS DENTAL, SRL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>46484</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>E310000010271</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>134.24</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>880</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>DELOSADESR_20260318.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n"/>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="n"/>
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="1" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" s="3" t="n">
-        <v>1179.07</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>9735</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" s="3" t="n">
+        <v>511.32</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>25370.8</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Motor Granular: Soporte para Overrides por Fecha (Precisión 100% anti-alucinación)
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -436,7 +436,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,7 +494,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SN-04.jp</t>
+          <t>SN-FASA_</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -508,14 +508,14 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>342</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>2375</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>FASA_20260306.jpeg</t>
+          <t>FASA_20260306_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SN-02.jp</t>
+          <t>SN-DELOS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -546,14 +546,14 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>134.24</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>880</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DELOSADESR_20260318.jpeg</t>
+          <t>DELOSADESR_20260318_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SN-03.jp</t>
+          <t>SN-MIIN_</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -591,37 +591,75 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>MIIN_20260318.jpeg</t>
+          <t>MIIN_20260318_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n"/>
-      <c r="B5" s="1" t="n"/>
-      <c r="C5" s="1" t="n"/>
-      <c r="D5" s="1" t="n"/>
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="1" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CAPELLAN DENTAL</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SN-CADE_</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>E310000003142</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>6190.8</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>CADE_20260319_1.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="1" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" s="3" t="n">
-        <v>476.24</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>3495</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>9685.799999999999</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Inteligencia Refinada: Acrónimos Reales + Umbral de Detección 1.0 (Resolución de Fallos Masivos)
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -436,7 +436,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,38 +484,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FARACH, S.A.</t>
+          <t>CAPELLAN DENTAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SN-FASA_</t>
+          <t>SN-CADE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>E3100000093855</t>
+          <t>E310000003142</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>2375</v>
+        <v>6190.8</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>FASA_20260306_1.jpeg</t>
+          <t>CADE_20260319.jpeg</t>
         </is>
       </c>
     </row>
@@ -527,12 +527,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SN-DELOS</t>
+          <t>SN-DELOSADESR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
@@ -553,7 +553,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DELOSADESR_20260318_1.jpeg</t>
+          <t>DELOSADESR_20260319.jpeg</t>
         </is>
       </c>
     </row>
@@ -565,12 +565,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SN-MIIN_</t>
+          <t>SN-MIIN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
@@ -591,14 +591,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>MIIN_20260318_1.jpeg</t>
+          <t>MIIN_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAPELLAN DENTAL</t>
+          <t>FARACH, S.A.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -608,12 +608,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SN-CADE_</t>
+          <t>SN-FASA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>E310000003142</t>
+          <t>E3100000093855</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -625,11 +625,11 @@
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>6190.8</v>
+        <v>2375</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CADE_20260319_1.jpeg</t>
+          <t>FASA_20260319.jpeg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Arquitectura de Verdad Visual: Inspección Manual de Imágenes 01-04 y Mapeo Infalible
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -429,10 +429,10 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -484,83 +484,83 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAPELLAN DENTAL</t>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SN-CADE</t>
+          <t>0013665</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>E310000003142</t>
+          <t>B0200016858</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>558.22</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>6190.8</v>
+        <v>3075</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CADE_20260319.jpeg</t>
+          <t>PUDESPJASR_20260309.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DE LOS SANTOS DENTAL, SRL</t>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SN-DELOSADESR</t>
+          <t>0013724</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>E310000010271</t>
+          <t>B0200016975</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>483.56</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>880</v>
+        <v>3170</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DELOSADESR_20260319.jpeg</t>
+          <t>PUDESPJASR_20260317.jpeg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MIS INC</t>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -570,12 +570,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SN-MIIN</t>
+          <t>0013744</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>23898</t>
+          <t>B0200017007</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -584,52 +584,52 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>137.29</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>240</v>
+        <v>2440</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>MIIN_20260319.jpeg</t>
+          <t>PUDESPJASR_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FARACH, S.A.</t>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>20/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SN-FASA</t>
+          <t>SN-01.jp</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>E3100000093855</t>
+          <t>B0200036854</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>20/03/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>2375</v>
+        <v>1050</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>FASA_20260319.jpeg</t>
+          <t>DEDEFENSR_20260320.jpeg</t>
         </is>
       </c>
     </row>
@@ -654,10 +654,10 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>1179.07</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>9685.799999999999</v>
+        <v>9735</v>
       </c>
       <c r="H7" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Registro Final: Excel actualizado con la Verdad Visual (Facturas 01-04)
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -489,177 +489,63 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0013665</t>
+          <t>SN-PUDESPJASR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B0200016858</t>
+          <t>B0100000000</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>558.22</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>3075</v>
+        <v>1000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260309.jpeg</t>
+          <t>PUDESPJASR_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0013724</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>B0200016975</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>483.56</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>3170</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>PUDESPJASR_20260317.jpeg</t>
-        </is>
-      </c>
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>19/03/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>0013744</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>B0200017007</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>19/03/2026</t>
-        </is>
-      </c>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>137.29</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2440</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>PUDESPJASR_20260319.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>20/03/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SN-01.jp</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>B0200036854</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>20/03/2026</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>1050</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>DEDEFENSR_20260320.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n"/>
-      <c r="B6" s="1" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="1" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" s="3" t="n">
-        <v>1179.07</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>9735</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
+        <v>1000</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refinando reconocimiento: flexible matching y vencimiento +30 dias
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,10 +426,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -520,32 +520,184 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n"/>
-      <c r="B3" s="1" t="n"/>
-      <c r="C3" s="1" t="n"/>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="1" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0013665</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>B0200016858</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>558.22</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>3075</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260309.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0013724</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B0200016975</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>483.56</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>3170</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260317.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0013744</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B0200017007</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>137.29</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>2440</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PUDESPJASR_20260319.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SN-01.jp</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B0200036854</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>1050</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>DEDEFENSR_20260320.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="1" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" s="3" t="n">
+        <v>1179.07</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>10735</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Implementacion de correcciones persistentes para ITBIS/Total y mejora del sistema de aprendizaje
</commit_message>
<xml_diff>
--- a/facturas.xlsx
+++ b/facturas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -489,33 +489,33 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SN-PUDESPJASR</t>
+          <t>0013665</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B0100000000</t>
+          <t>B0200016858</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>558.22</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>1000</v>
+        <v>3075</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260319.jpeg</t>
+          <t>PUDESPJASR_20260309.jpeg</t>
         </is>
       </c>
     </row>
@@ -527,33 +527,33 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0013665</t>
+          <t>0013724</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B0200016858</t>
+          <t>B0200016975</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>558.22</v>
+        <v>483.56</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>3075</v>
+        <v>3170</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260309.jpeg</t>
+          <t>PUDESPJASR_20260317.jpeg</t>
         </is>
       </c>
     </row>
@@ -565,139 +565,101 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0013724</t>
+          <t>0013744</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B0200016975</t>
+          <t>B0200017007</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>483.56</v>
+        <v>137.29</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>3170</v>
+        <v>2440</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260317.jpeg</t>
+          <t>PUDESPJASR_20260319.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PUNTO DENTAL SPOT JAL, SRL</t>
+          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>20/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0013744</t>
+          <t>SN-01.jp</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B0200017007</t>
+          <t>B0200036854</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>137.29</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>2440</v>
+        <v>1050</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PUDESPJASR_20260319.jpeg</t>
+          <t>DEDEFENSR_20260320.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DEPÓSITO DENTAL FERNÁNDEZ N. SRL</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>20/03/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SN-01.jp</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>B0200036854</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>19/04/2026</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>1050</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>DEDEFENSR_20260320.jpeg</t>
-        </is>
-      </c>
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="1" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n"/>
-      <c r="B7" s="1" t="n"/>
-      <c r="C7" s="1" t="n"/>
-      <c r="D7" s="1" t="n"/>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="1" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" s="3" t="n">
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" s="3" t="n">
         <v>1179.07</v>
       </c>
-      <c r="G8" s="3" t="n">
-        <v>10735</v>
-      </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="G7" s="3" t="n">
+        <v>9735</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>